<commit_message>
make_results_excel: add StableVSR baseline (3 methods x 4 datasets)
</commit_message>
<xml_diff>
--- a/results_comparison.xlsx
+++ b/results_comparison.xlsx
@@ -161,16 +161,16 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -542,7 +542,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -656,585 +656,721 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>BasicVSR++</t>
+          <t>StableVSR (baseline)</t>
         </is>
       </c>
       <c r="B4" s="9" t="n">
-        <v>24.88</v>
+        <v>24.04</v>
       </c>
       <c r="C4" s="10" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>0.364</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>0.179</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>41.23</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>0.265</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="I4" s="12" t="n">
-        <v>38.26</v>
-      </c>
-      <c r="J4" s="11" t="n">
-        <v>13.739</v>
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>42.79</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>0.237</v>
+      </c>
+      <c r="H4" s="10" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>41.11</v>
+      </c>
+      <c r="J4" s="10" t="n">
+        <v>13.962</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
+          <t>BasicVSR++</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>41.23</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>38.26</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>13.739</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
           <t>Ours (dual-SFT)</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B6" s="9" t="n">
         <v>24.48</v>
       </c>
-      <c r="C5" s="11" t="n">
+      <c r="C6" s="10" t="n">
         <v>0.6909999999999999</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D6" s="12" t="n">
         <v>0.193</v>
       </c>
-      <c r="E5" s="10" t="n">
+      <c r="E6" s="12" t="n">
         <v>0.08799999999999999</v>
       </c>
-      <c r="F5" s="9" t="n">
+      <c r="F6" s="11" t="n">
         <v>65.7</v>
       </c>
-      <c r="G5" s="10" t="n">
+      <c r="G6" s="12" t="n">
         <v>0.386</v>
       </c>
-      <c r="H5" s="10" t="n">
+      <c r="H6" s="12" t="n">
         <v>2.77</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I6" s="11" t="n">
         <v>15.25</v>
       </c>
-      <c r="J5" s="10" t="n">
+      <c r="J6" s="12" t="n">
         <v>11.12</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="1" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Vid4</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="3" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="B8" s="2" t="n"/>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+      <c r="F8" s="2" t="n"/>
+      <c r="G8" s="2" t="n"/>
+      <c r="H8" s="2" t="n"/>
+      <c r="I8" s="2" t="n"/>
+      <c r="J8" s="3" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>Reconstruction</t>
         </is>
       </c>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="C9" s="5" t="n"/>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Reference Perceptual</t>
         </is>
       </c>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="E9" s="5" t="n"/>
+      <c r="F9" s="4" t="inlineStr">
         <is>
           <t>No-reference Perceptual</t>
         </is>
       </c>
-      <c r="G8" s="5" t="n"/>
-      <c r="H8" s="5" t="n"/>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="G9" s="5" t="n"/>
+      <c r="H9" s="5" t="n"/>
+      <c r="I9" s="4" t="inlineStr">
         <is>
           <t>Temporal</t>
         </is>
       </c>
-      <c r="J8" s="5" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr"/>
-      <c r="B9" s="7" t="inlineStr">
+      <c r="J9" s="5" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>PSNR ↑</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C10" s="7" t="inlineStr">
         <is>
           <t>SSIM ↑</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>LPIPS ↓</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E10" s="7" t="inlineStr">
         <is>
           <t>DISTS ↓</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>MUSIQ ↑</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>CLIP-IQA ↑</t>
         </is>
       </c>
-      <c r="H9" s="7" t="inlineStr">
+      <c r="H10" s="7" t="inlineStr">
         <is>
           <t>NIQE ↓</t>
         </is>
       </c>
-      <c r="I9" s="7" t="inlineStr">
+      <c r="I10" s="7" t="inlineStr">
         <is>
           <t>tLPIPS ↓</t>
         </is>
       </c>
-      <c r="J9" s="7" t="inlineStr">
+      <c r="J10" s="7" t="inlineStr">
         <is>
           <t>tOF ↓</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>BasicVSR++</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="n">
-        <v>26.26</v>
-      </c>
-      <c r="C10" s="10" t="n">
-        <v>0.828</v>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="E10" s="11" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="F10" s="12" t="n">
-        <v>61.5</v>
-      </c>
-      <c r="G10" s="11" t="n">
-        <v>0.341</v>
-      </c>
-      <c r="H10" s="11" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="I10" s="9" t="n">
-        <v>15.12</v>
-      </c>
-      <c r="J10" s="10" t="n">
-        <v>0.489</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
+          <t>StableVSR (baseline)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>22.98</v>
+      </c>
+      <c r="C11" s="10" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="D11" s="12" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="E11" s="12" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>67.22</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="H11" s="12" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="I11" s="9" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="J11" s="10" t="n">
+        <v>0.751</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>BasicVSR++</t>
+        </is>
+      </c>
+      <c r="B12" s="11" t="n">
+        <v>26.26</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.341</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="I12" s="11" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="J12" s="12" t="n">
+        <v>0.489</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
           <t>Ours (dual-SFT)</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B13" s="9" t="n">
         <v>22.64</v>
       </c>
-      <c r="C11" s="11" t="n">
+      <c r="C13" s="10" t="n">
         <v>0.664</v>
       </c>
-      <c r="D11" s="11" t="n">
+      <c r="D13" s="10" t="n">
         <v>0.194</v>
       </c>
-      <c r="E11" s="10" t="n">
+      <c r="E13" s="10" t="n">
         <v>0.114</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F13" s="9" t="n">
         <v>66.15000000000001</v>
       </c>
-      <c r="G11" s="10" t="n">
+      <c r="G13" s="10" t="n">
         <v>0.408</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H13" s="10" t="n">
         <v>3.32</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I13" s="9" t="n">
         <v>28.53</v>
       </c>
-      <c r="J11" s="11" t="n">
+      <c r="J13" s="10" t="n">
         <v>0.92</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
         <is>
           <t>UDM10</t>
         </is>
       </c>
-      <c r="B13" s="2" t="n"/>
-      <c r="C13" s="2" t="n"/>
-      <c r="D13" s="2" t="n"/>
-      <c r="E13" s="2" t="n"/>
-      <c r="F13" s="2" t="n"/>
-      <c r="G13" s="2" t="n"/>
-      <c r="H13" s="2" t="n"/>
-      <c r="I13" s="2" t="n"/>
-      <c r="J13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="n"/>
+      <c r="G15" s="2" t="n"/>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="3" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B16" s="4" t="inlineStr">
         <is>
           <t>Reconstruction</t>
         </is>
       </c>
-      <c r="C14" s="5" t="n"/>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="C16" s="5" t="n"/>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>Reference Perceptual</t>
         </is>
       </c>
-      <c r="E14" s="5" t="n"/>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="E16" s="5" t="n"/>
+      <c r="F16" s="4" t="inlineStr">
         <is>
           <t>No-reference Perceptual</t>
         </is>
       </c>
-      <c r="G14" s="5" t="n"/>
-      <c r="H14" s="5" t="n"/>
-      <c r="I14" s="4" t="inlineStr">
+      <c r="G16" s="5" t="n"/>
+      <c r="H16" s="5" t="n"/>
+      <c r="I16" s="4" t="inlineStr">
         <is>
           <t>Temporal</t>
         </is>
       </c>
-      <c r="J14" s="5" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr"/>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="J16" s="5" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr"/>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>PSNR ↑</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>SSIM ↑</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>LPIPS ↓</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>DISTS ↓</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>MUSIQ ↑</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>CLIP-IQA ↑</t>
         </is>
       </c>
-      <c r="H15" s="7" t="inlineStr">
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>NIQE ↓</t>
         </is>
       </c>
-      <c r="I15" s="7" t="inlineStr">
+      <c r="I17" s="7" t="inlineStr">
         <is>
           <t>tLPIPS ↓</t>
         </is>
       </c>
-      <c r="J15" s="7" t="inlineStr">
+      <c r="J17" s="7" t="inlineStr">
         <is>
           <t>tOF ↓</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>StableVSR (baseline)</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="F18" s="9" t="n">
+        <v>55.69</v>
+      </c>
+      <c r="G18" s="10" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="H18" s="10" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="I18" s="11" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="J18" s="10" t="n">
+        <v>1.828</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
         <is>
           <t>BasicVSR++</t>
         </is>
       </c>
-      <c r="B16" s="9" t="n">
+      <c r="B19" s="11" t="n">
         <v>37.48</v>
       </c>
-      <c r="C16" s="10" t="n">
+      <c r="C19" s="12" t="n">
         <v>0.956</v>
       </c>
-      <c r="D16" s="10" t="n">
+      <c r="D19" s="12" t="n">
         <v>0.06</v>
       </c>
-      <c r="E16" s="10" t="n">
+      <c r="E19" s="12" t="n">
         <v>0.053</v>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F19" s="9" t="n">
         <v>59.36</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G19" s="10" t="n">
         <v>0.443</v>
       </c>
-      <c r="H16" s="11" t="n">
+      <c r="H19" s="10" t="n">
         <v>5.6</v>
       </c>
-      <c r="I16" s="9" t="n">
+      <c r="I19" s="9" t="n">
         <v>5.55</v>
       </c>
-      <c r="J16" s="10" t="n">
+      <c r="J19" s="12" t="n">
         <v>1.191</v>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
         <is>
           <t>Ours (dual-SFT)</t>
         </is>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B20" s="9" t="n">
         <v>25.54</v>
       </c>
-      <c r="C17" s="11" t="n">
+      <c r="C20" s="10" t="n">
         <v>0.8110000000000001</v>
       </c>
-      <c r="D17" s="11" t="n">
+      <c r="D20" s="10" t="n">
         <v>0.124</v>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E20" s="10" t="n">
         <v>0.066</v>
       </c>
-      <c r="F17" s="9" t="n">
+      <c r="F20" s="11" t="n">
         <v>63.2</v>
       </c>
-      <c r="G17" s="10" t="n">
+      <c r="G20" s="12" t="n">
         <v>0.447</v>
       </c>
-      <c r="H17" s="10" t="n">
+      <c r="H20" s="12" t="n">
         <v>4.12</v>
       </c>
-      <c r="I17" s="12" t="n">
+      <c r="I20" s="9" t="n">
         <v>14.48</v>
       </c>
-      <c r="J17" s="11" t="n">
+      <c r="J20" s="10" t="n">
         <v>2.518</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="1" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="1" t="inlineStr">
         <is>
           <t>SPMCS</t>
         </is>
       </c>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
-      <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="3" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="3" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="4" t="inlineStr">
         <is>
           <t>Method</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>Reconstruction</t>
         </is>
       </c>
-      <c r="C20" s="5" t="n"/>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="C23" s="5" t="n"/>
+      <c r="D23" s="4" t="inlineStr">
         <is>
           <t>Reference Perceptual</t>
         </is>
       </c>
-      <c r="E20" s="5" t="n"/>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="E23" s="5" t="n"/>
+      <c r="F23" s="4" t="inlineStr">
         <is>
           <t>No-reference Perceptual</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n"/>
-      <c r="H20" s="5" t="n"/>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="G23" s="5" t="n"/>
+      <c r="H23" s="5" t="n"/>
+      <c r="I23" s="4" t="inlineStr">
         <is>
           <t>Temporal</t>
         </is>
       </c>
-      <c r="J20" s="5" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr"/>
-      <c r="B21" s="7" t="inlineStr">
+      <c r="J23" s="5" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr"/>
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>PSNR ↑</t>
         </is>
       </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C24" s="7" t="inlineStr">
         <is>
           <t>SSIM ↑</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D24" s="7" t="inlineStr">
         <is>
           <t>LPIPS ↓</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E24" s="7" t="inlineStr">
         <is>
           <t>DISTS ↓</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
+      <c r="F24" s="7" t="inlineStr">
         <is>
           <t>MUSIQ ↑</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr">
+      <c r="G24" s="7" t="inlineStr">
         <is>
           <t>CLIP-IQA ↑</t>
         </is>
       </c>
-      <c r="H21" s="7" t="inlineStr">
+      <c r="H24" s="7" t="inlineStr">
         <is>
           <t>NIQE ↓</t>
         </is>
       </c>
-      <c r="I21" s="7" t="inlineStr">
+      <c r="I24" s="7" t="inlineStr">
         <is>
           <t>tLPIPS ↓</t>
         </is>
       </c>
-      <c r="J21" s="7" t="inlineStr">
+      <c r="J24" s="7" t="inlineStr">
         <is>
           <t>tOF ↓</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr">
+        <is>
+          <t>StableVSR (baseline)</t>
+        </is>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>19.42</v>
+      </c>
+      <c r="C25" s="10" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="D25" s="10" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="E25" s="10" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="F25" s="11" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="G25" s="12" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="H25" s="12" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="I25" s="9" t="n">
+        <v>51.11</v>
+      </c>
+      <c r="J25" s="10" t="n">
+        <v>0.652</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>BasicVSR++</t>
         </is>
       </c>
-      <c r="B22" s="9" t="n">
+      <c r="B26" s="11" t="n">
         <v>21.94</v>
       </c>
-      <c r="C22" s="10" t="n">
+      <c r="C26" s="12" t="n">
         <v>0.617</v>
       </c>
-      <c r="D22" s="11" t="n">
+      <c r="D26" s="10" t="n">
         <v>0.187</v>
       </c>
-      <c r="E22" s="11" t="n">
+      <c r="E26" s="10" t="n">
         <v>0.108</v>
       </c>
-      <c r="F22" s="12" t="n">
+      <c r="F26" s="9" t="n">
         <v>62.48</v>
       </c>
-      <c r="G22" s="11" t="n">
+      <c r="G26" s="10" t="n">
         <v>0.434</v>
       </c>
-      <c r="H22" s="11" t="n">
+      <c r="H26" s="10" t="n">
         <v>5.17</v>
       </c>
-      <c r="I22" s="9" t="n">
+      <c r="I26" s="11" t="n">
         <v>3.6</v>
       </c>
-      <c r="J22" s="10" t="n">
+      <c r="J26" s="12" t="n">
         <v>0.345</v>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
         <is>
           <t>Ours (dual-SFT)</t>
         </is>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B27" s="9" t="n">
         <v>19.94</v>
       </c>
-      <c r="C23" s="11" t="n">
+      <c r="C27" s="10" t="n">
         <v>0.506</v>
       </c>
-      <c r="D23" s="10" t="n">
+      <c r="D27" s="12" t="n">
         <v>0.183</v>
       </c>
-      <c r="E23" s="10" t="n">
+      <c r="E27" s="12" t="n">
         <v>0.106</v>
       </c>
-      <c r="F23" s="9" t="n">
+      <c r="F27" s="9" t="n">
         <v>67.22</v>
       </c>
-      <c r="G23" s="10" t="n">
+      <c r="G27" s="10" t="n">
         <v>0.503</v>
       </c>
-      <c r="H23" s="10" t="n">
+      <c r="H27" s="10" t="n">
         <v>3.7</v>
       </c>
-      <c r="I23" s="12" t="n">
+      <c r="I27" s="9" t="n">
         <v>31.59</v>
       </c>
-      <c r="J23" s="11" t="n">
+      <c r="J27" s="10" t="n">
         <v>0.576</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="B16:C16"/>
+    <mergeCell ref="A8:J8"/>
+    <mergeCell ref="A22:J22"/>
     <mergeCell ref="I2:J2"/>
-    <mergeCell ref="F8:H8"/>
     <mergeCell ref="F2:H2"/>
-    <mergeCell ref="A19:J19"/>
-    <mergeCell ref="A13:J13"/>
+    <mergeCell ref="F23:H23"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D2:E2"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="B8:C8"/>
+    <mergeCell ref="I16:J16"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A15:J15"/>
+    <mergeCell ref="F9:H9"/>
     <mergeCell ref="A1:J1"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="A7:J7"/>
-    <mergeCell ref="I14:J14"/>
-    <mergeCell ref="I8:J8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="I20:J20"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="I23:J23"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F16:H16"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="I9:J9"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1246,7 +1382,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J15"/>
+  <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1264,7 +1400,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BasicVSR++</t>
+          <t>StableVSR (baseline)</t>
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
@@ -1363,32 +1499,32 @@
           <t>REDS4</t>
         </is>
       </c>
-      <c r="B4" s="12" t="n">
-        <v>24.88</v>
-      </c>
-      <c r="C4" s="11" t="n">
-        <v>0.73</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>0.364</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>0.179</v>
-      </c>
-      <c r="F4" s="12" t="n">
-        <v>41.23</v>
-      </c>
-      <c r="G4" s="11" t="n">
-        <v>0.265</v>
-      </c>
-      <c r="H4" s="11" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="I4" s="12" t="n">
-        <v>38.26</v>
-      </c>
-      <c r="J4" s="11" t="n">
-        <v>13.739</v>
+      <c r="B4" s="9" t="n">
+        <v>24.04</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="D4" s="10" t="n">
+        <v>0.309</v>
+      </c>
+      <c r="E4" s="10" t="n">
+        <v>0.164</v>
+      </c>
+      <c r="F4" s="9" t="n">
+        <v>42.79</v>
+      </c>
+      <c r="G4" s="10" t="n">
+        <v>0.237</v>
+      </c>
+      <c r="H4" s="10" t="n">
+        <v>4.38</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>41.11</v>
+      </c>
+      <c r="J4" s="10" t="n">
+        <v>13.962</v>
       </c>
     </row>
     <row r="5">
@@ -1397,32 +1533,32 @@
           <t>Vid4</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
-        <v>26.26</v>
-      </c>
-      <c r="C5" s="11" t="n">
-        <v>0.828</v>
-      </c>
-      <c r="D5" s="11" t="n">
-        <v>0.189</v>
-      </c>
-      <c r="E5" s="11" t="n">
-        <v>0.122</v>
-      </c>
-      <c r="F5" s="12" t="n">
-        <v>61.5</v>
-      </c>
-      <c r="G5" s="11" t="n">
-        <v>0.341</v>
-      </c>
-      <c r="H5" s="11" t="n">
-        <v>5.04</v>
-      </c>
-      <c r="I5" s="12" t="n">
-        <v>15.12</v>
-      </c>
-      <c r="J5" s="11" t="n">
-        <v>0.489</v>
+      <c r="B5" s="9" t="n">
+        <v>22.98</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0.674</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.185</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>0.107</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>67.22</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>0.454</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>3.19</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>25.36</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>0.751</v>
       </c>
     </row>
     <row r="6">
@@ -1431,32 +1567,32 @@
           <t>UDM10</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
-        <v>37.48</v>
-      </c>
-      <c r="C6" s="11" t="n">
-        <v>0.956</v>
-      </c>
-      <c r="D6" s="11" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="E6" s="11" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="F6" s="12" t="n">
-        <v>59.36</v>
-      </c>
-      <c r="G6" s="11" t="n">
-        <v>0.443</v>
-      </c>
-      <c r="H6" s="11" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="I6" s="12" t="n">
-        <v>5.55</v>
-      </c>
-      <c r="J6" s="11" t="n">
-        <v>1.191</v>
+      <c r="B6" s="9" t="n">
+        <v>26.71</v>
+      </c>
+      <c r="C6" s="10" t="n">
+        <v>0.834</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0.055</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>55.69</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>0.362</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>4.66</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>4.42</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>1.828</v>
       </c>
     </row>
     <row r="7">
@@ -1465,38 +1601,38 @@
           <t>SPMCS</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
-        <v>21.94</v>
-      </c>
-      <c r="C7" s="11" t="n">
-        <v>0.617</v>
-      </c>
-      <c r="D7" s="11" t="n">
-        <v>0.187</v>
-      </c>
-      <c r="E7" s="11" t="n">
-        <v>0.108</v>
-      </c>
-      <c r="F7" s="12" t="n">
-        <v>62.48</v>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>0.434</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>5.17</v>
-      </c>
-      <c r="I7" s="12" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <v>0.345</v>
+      <c r="B7" s="9" t="n">
+        <v>19.42</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.478</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.196</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>0.112</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>69.98</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0.582</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>3.28</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>51.11</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>0.652</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Ours (dual-SFT)</t>
+          <t>BasicVSR++</t>
         </is>
       </c>
       <c r="B9" s="2" t="n"/>
@@ -1595,32 +1731,32 @@
           <t>REDS4</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
-        <v>24.48</v>
-      </c>
-      <c r="C12" s="11" t="n">
-        <v>0.6909999999999999</v>
-      </c>
-      <c r="D12" s="11" t="n">
-        <v>0.193</v>
-      </c>
-      <c r="E12" s="11" t="n">
-        <v>0.08799999999999999</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>65.7</v>
-      </c>
-      <c r="G12" s="11" t="n">
-        <v>0.386</v>
-      </c>
-      <c r="H12" s="11" t="n">
-        <v>2.77</v>
-      </c>
-      <c r="I12" s="12" t="n">
-        <v>15.25</v>
-      </c>
-      <c r="J12" s="11" t="n">
-        <v>11.12</v>
+      <c r="B12" s="9" t="n">
+        <v>24.88</v>
+      </c>
+      <c r="C12" s="10" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="D12" s="10" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>0.179</v>
+      </c>
+      <c r="F12" s="9" t="n">
+        <v>41.23</v>
+      </c>
+      <c r="G12" s="10" t="n">
+        <v>0.265</v>
+      </c>
+      <c r="H12" s="10" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="I12" s="9" t="n">
+        <v>38.26</v>
+      </c>
+      <c r="J12" s="10" t="n">
+        <v>13.739</v>
       </c>
     </row>
     <row r="13">
@@ -1629,32 +1765,32 @@
           <t>Vid4</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
-        <v>22.64</v>
-      </c>
-      <c r="C13" s="11" t="n">
-        <v>0.664</v>
-      </c>
-      <c r="D13" s="11" t="n">
-        <v>0.194</v>
-      </c>
-      <c r="E13" s="11" t="n">
-        <v>0.114</v>
-      </c>
-      <c r="F13" s="12" t="n">
-        <v>66.15000000000001</v>
-      </c>
-      <c r="G13" s="11" t="n">
-        <v>0.408</v>
-      </c>
-      <c r="H13" s="11" t="n">
-        <v>3.32</v>
-      </c>
-      <c r="I13" s="12" t="n">
-        <v>28.53</v>
-      </c>
-      <c r="J13" s="11" t="n">
-        <v>0.92</v>
+      <c r="B13" s="9" t="n">
+        <v>26.26</v>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>0.828</v>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>0.189</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>0.122</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>61.5</v>
+      </c>
+      <c r="G13" s="10" t="n">
+        <v>0.341</v>
+      </c>
+      <c r="H13" s="10" t="n">
+        <v>5.04</v>
+      </c>
+      <c r="I13" s="9" t="n">
+        <v>15.12</v>
+      </c>
+      <c r="J13" s="10" t="n">
+        <v>0.489</v>
       </c>
     </row>
     <row r="14">
@@ -1663,32 +1799,32 @@
           <t>UDM10</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
-        <v>25.54</v>
-      </c>
-      <c r="C14" s="11" t="n">
-        <v>0.8110000000000001</v>
-      </c>
-      <c r="D14" s="11" t="n">
-        <v>0.124</v>
-      </c>
-      <c r="E14" s="11" t="n">
-        <v>0.066</v>
-      </c>
-      <c r="F14" s="12" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="G14" s="11" t="n">
-        <v>0.447</v>
-      </c>
-      <c r="H14" s="11" t="n">
-        <v>4.12</v>
-      </c>
-      <c r="I14" s="12" t="n">
-        <v>14.48</v>
-      </c>
-      <c r="J14" s="11" t="n">
-        <v>2.518</v>
+      <c r="B14" s="9" t="n">
+        <v>37.48</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0.956</v>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>0.053</v>
+      </c>
+      <c r="F14" s="9" t="n">
+        <v>59.36</v>
+      </c>
+      <c r="G14" s="10" t="n">
+        <v>0.443</v>
+      </c>
+      <c r="H14" s="10" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="I14" s="9" t="n">
+        <v>5.55</v>
+      </c>
+      <c r="J14" s="10" t="n">
+        <v>1.191</v>
       </c>
     </row>
     <row r="15">
@@ -1697,46 +1833,283 @@
           <t>SPMCS</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="9" t="n">
+        <v>21.94</v>
+      </c>
+      <c r="C15" s="10" t="n">
+        <v>0.617</v>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>0.187</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>0.108</v>
+      </c>
+      <c r="F15" s="9" t="n">
+        <v>62.48</v>
+      </c>
+      <c r="G15" s="10" t="n">
+        <v>0.434</v>
+      </c>
+      <c r="H15" s="10" t="n">
+        <v>5.17</v>
+      </c>
+      <c r="I15" s="9" t="n">
+        <v>3.6</v>
+      </c>
+      <c r="J15" s="10" t="n">
+        <v>0.345</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Ours (dual-SFT)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+      <c r="C17" s="2" t="n"/>
+      <c r="D17" s="2" t="n"/>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="n"/>
+      <c r="G17" s="2" t="n"/>
+      <c r="H17" s="2" t="n"/>
+      <c r="I17" s="2" t="n"/>
+      <c r="J17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Dataset</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Reconstruction</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="n"/>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Reference Perceptual</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="n"/>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>No-reference Perceptual</t>
+        </is>
+      </c>
+      <c r="G18" s="5" t="n"/>
+      <c r="H18" s="5" t="n"/>
+      <c r="I18" s="4" t="inlineStr">
+        <is>
+          <t>Temporal</t>
+        </is>
+      </c>
+      <c r="J18" s="5" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>PSNR ↑</t>
+        </is>
+      </c>
+      <c r="C19" s="7" t="inlineStr">
+        <is>
+          <t>SSIM ↑</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>LPIPS ↓</t>
+        </is>
+      </c>
+      <c r="E19" s="7" t="inlineStr">
+        <is>
+          <t>DISTS ↓</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr">
+        <is>
+          <t>MUSIQ ↑</t>
+        </is>
+      </c>
+      <c r="G19" s="7" t="inlineStr">
+        <is>
+          <t>CLIP-IQA ↑</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
+        <is>
+          <t>NIQE ↓</t>
+        </is>
+      </c>
+      <c r="I19" s="7" t="inlineStr">
+        <is>
+          <t>tLPIPS ↓</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
+          <t>tOF ↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="13" t="inlineStr">
+        <is>
+          <t>REDS4</t>
+        </is>
+      </c>
+      <c r="B20" s="9" t="n">
+        <v>24.48</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="D20" s="10" t="n">
+        <v>0.193</v>
+      </c>
+      <c r="E20" s="10" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="F20" s="9" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="G20" s="10" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="H20" s="10" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="I20" s="9" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="J20" s="10" t="n">
+        <v>11.12</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="13" t="inlineStr">
+        <is>
+          <t>Vid4</t>
+        </is>
+      </c>
+      <c r="B21" s="9" t="n">
+        <v>22.64</v>
+      </c>
+      <c r="C21" s="10" t="n">
+        <v>0.664</v>
+      </c>
+      <c r="D21" s="10" t="n">
+        <v>0.194</v>
+      </c>
+      <c r="E21" s="10" t="n">
+        <v>0.114</v>
+      </c>
+      <c r="F21" s="9" t="n">
+        <v>66.15000000000001</v>
+      </c>
+      <c r="G21" s="10" t="n">
+        <v>0.408</v>
+      </c>
+      <c r="H21" s="10" t="n">
+        <v>3.32</v>
+      </c>
+      <c r="I21" s="9" t="n">
+        <v>28.53</v>
+      </c>
+      <c r="J21" s="10" t="n">
+        <v>0.92</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>UDM10</t>
+        </is>
+      </c>
+      <c r="B22" s="9" t="n">
+        <v>25.54</v>
+      </c>
+      <c r="C22" s="10" t="n">
+        <v>0.8110000000000001</v>
+      </c>
+      <c r="D22" s="10" t="n">
+        <v>0.124</v>
+      </c>
+      <c r="E22" s="10" t="n">
+        <v>0.066</v>
+      </c>
+      <c r="F22" s="9" t="n">
+        <v>63.2</v>
+      </c>
+      <c r="G22" s="10" t="n">
+        <v>0.447</v>
+      </c>
+      <c r="H22" s="10" t="n">
+        <v>4.12</v>
+      </c>
+      <c r="I22" s="9" t="n">
+        <v>14.48</v>
+      </c>
+      <c r="J22" s="10" t="n">
+        <v>2.518</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>SPMCS</t>
+        </is>
+      </c>
+      <c r="B23" s="9" t="n">
         <v>19.94</v>
       </c>
-      <c r="C15" s="11" t="n">
+      <c r="C23" s="10" t="n">
         <v>0.506</v>
       </c>
-      <c r="D15" s="11" t="n">
+      <c r="D23" s="10" t="n">
         <v>0.183</v>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E23" s="10" t="n">
         <v>0.106</v>
       </c>
-      <c r="F15" s="12" t="n">
+      <c r="F23" s="9" t="n">
         <v>67.22</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G23" s="10" t="n">
         <v>0.503</v>
       </c>
-      <c r="H15" s="11" t="n">
+      <c r="H23" s="10" t="n">
         <v>3.7</v>
       </c>
-      <c r="I15" s="12" t="n">
+      <c r="I23" s="9" t="n">
         <v>31.59</v>
       </c>
-      <c r="J15" s="11" t="n">
+      <c r="J23" s="10" t="n">
         <v>0.576</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="15">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="F10:H10"/>
     <mergeCell ref="B2:C2"/>
     <mergeCell ref="D10:E10"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F18:H18"/>
+    <mergeCell ref="A17:J17"/>
     <mergeCell ref="A9:J9"/>
     <mergeCell ref="I2:J2"/>
     <mergeCell ref="I10:J10"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="F2:H2"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="I18:J18"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Excel: add Ablation (REDS4) sheet with 4 inference-time variants
</commit_message>
<xml_diff>
--- a/results_comparison.xlsx
+++ b/results_comparison.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet name="By Dataset" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="By Method" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Notes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ablation (REDS4)" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Notes" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2121,7 +2122,272 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A26"/>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Inference-time Ablation on REDS4</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="3" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr">
+        <is>
+          <t>Variant</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Reconstruction</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n"/>
+      <c r="D2" s="4" t="inlineStr">
+        <is>
+          <t>Reference Perceptual</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="n"/>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>No-reference Perceptual</t>
+        </is>
+      </c>
+      <c r="G2" s="5" t="n"/>
+      <c r="H2" s="5" t="n"/>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Temporal</t>
+        </is>
+      </c>
+      <c r="J2" s="5" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr"/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>PSNR ↑</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>SSIM ↑</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>LPIPS ↓</t>
+        </is>
+      </c>
+      <c r="E3" s="7" t="inlineStr">
+        <is>
+          <t>DISTS ↓</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>MUSIQ ↑</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>CLIP-IQA ↑</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>NIQE ↓</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>tLPIPS ↓</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>tOF ↓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Ours full</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="n">
+        <v>24.48</v>
+      </c>
+      <c r="C4" s="10" t="n">
+        <v>0.6909999999999999</v>
+      </c>
+      <c r="D4" s="12" t="n">
+        <v>0.193</v>
+      </c>
+      <c r="E4" s="12" t="n">
+        <v>0.08799999999999999</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="G4" s="12" t="n">
+        <v>0.386</v>
+      </c>
+      <c r="H4" s="12" t="n">
+        <v>2.77</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <v>15.25</v>
+      </c>
+      <c r="J4" s="12" t="n">
+        <v>11.12</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="13" t="inlineStr">
+        <is>
+          <t>w/o HIGH</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="n">
+        <v>24.34</v>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0.6889999999999999</v>
+      </c>
+      <c r="D5" s="10" t="n">
+        <v>0.223</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>0.104</v>
+      </c>
+      <c r="F5" s="9" t="n">
+        <v>64.48999999999999</v>
+      </c>
+      <c r="G5" s="10" t="n">
+        <v>0.365</v>
+      </c>
+      <c r="H5" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>22.11</v>
+      </c>
+      <c r="J5" s="10" t="n">
+        <v>11.984</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>w/o LOW</t>
+        </is>
+      </c>
+      <c r="B6" s="11" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>0.701</v>
+      </c>
+      <c r="D6" s="10" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>0.098</v>
+      </c>
+      <c r="F6" s="9" t="n">
+        <v>63.39</v>
+      </c>
+      <c r="G6" s="10" t="n">
+        <v>0.335</v>
+      </c>
+      <c r="H6" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>16.57</v>
+      </c>
+      <c r="J6" s="10" t="n">
+        <v>11.392</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="13" t="inlineStr">
+        <is>
+          <t>w/o both</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="n">
+        <v>24.46</v>
+      </c>
+      <c r="C7" s="10" t="n">
+        <v>0.695</v>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>0.247</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>0.119</v>
+      </c>
+      <c r="F7" s="9" t="n">
+        <v>59.35</v>
+      </c>
+      <c r="G7" s="10" t="n">
+        <v>0.298</v>
+      </c>
+      <c r="H7" s="10" t="n">
+        <v>3.29</v>
+      </c>
+      <c r="I7" s="9" t="n">
+        <v>25.18</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>12.278</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:J1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="F2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -2283,9 +2549,75 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  - BasicVSR++ values for REDS4 / UDM10 not measured here; add if needed.</t>
+      <c r="A26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Ablation (REDS4, inference-time disabling):</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 'w/o HIGH': replace high_gamma=1, high_beta=0 (up_blocks[1] passthrough)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 'w/o LOW' : replace low_gamma=1,  low_beta=0  (down_blocks[1] passthrough)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  - 'w/o both': both disabled (both injection points are passthrough)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Interpretation:</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    * HIGH disabled hurts temporal stability (tLPIPS +45%) most</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    * LOW disabled hurts naturalness (MUSIQ, CLIP-IQA) most</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    * Both disabled is consistently worst on perceptual metrics</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    * w/o LOW slightly improves PSNR/SSIM (perceptual-distortion trade-off)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    * Synergy: LPIPS w/o-both (0.247) &gt; w/o-HIGH (0.223) + w/o-LOW (0.210) bias</t>
         </is>
       </c>
     </row>

</xml_diff>